<commit_message>
docs/tables: commit the outstanding regenerated results
- summary_all_objects_accuracy_f1{,_EN}.xlsx: alignment RMSE measured from the
  aligned clouds the site actually uses, plus 3/5/10cm and the delta column
- frame_count_study_summary.{json,xlsx}: rebuilt after the information_sign
  DBSCAN retune (ft7/eps3/mp5 -> ft5/eps2/mp3)
- registration_rmse_from_aligned_clouds.json: the RMSE those tables read
- icp_rmse_by_experiment.json: the earlier per-experiment ICP RMSE, kept for
  provenance (superseded by the file above, which measures the current clouds)
- records the two files deleted before this session (bus_stop_001 csv/summary,
  superseded by the xlsx and by the all-objects table)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tables/frame_count_study_summary.xlsx
+++ b/docs/tables/frame_count_study_summary.xlsx
@@ -594,22 +594,22 @@
         <v>27.08</v>
       </c>
       <c r="N2" t="n">
-        <v>34.85</v>
+        <v>35.36</v>
       </c>
       <c r="O2" t="n">
-        <v>47.76</v>
+        <v>47.64</v>
       </c>
       <c r="P2" t="n">
-        <v>83.31999999999999</v>
+        <v>83.22</v>
       </c>
       <c r="Q2" t="n">
-        <v>92.55</v>
+        <v>92.56999999999999</v>
       </c>
       <c r="R2" t="n">
-        <v>21.78</v>
+        <v>22.12</v>
       </c>
       <c r="S2" t="n">
-        <v>32.81</v>
+        <v>32.56</v>
       </c>
       <c r="T2" t="n">
         <v>1.33</v>
@@ -662,22 +662,22 @@
         <v>71.22</v>
       </c>
       <c r="N3" t="n">
-        <v>76.68000000000001</v>
+        <v>76.38</v>
       </c>
       <c r="O3" t="n">
-        <v>83.22</v>
+        <v>83.25</v>
       </c>
       <c r="P3" t="n">
-        <v>87.86</v>
+        <v>87.8</v>
       </c>
       <c r="Q3" t="n">
-        <v>94.41</v>
+        <v>94.45</v>
       </c>
       <c r="R3" t="n">
-        <v>66.45</v>
+        <v>66.04000000000001</v>
       </c>
       <c r="S3" t="n">
-        <v>75.97</v>
+        <v>75.76000000000001</v>
       </c>
       <c r="T3" t="n">
         <v>1.214</v>
@@ -730,22 +730,22 @@
         <v>77.51000000000001</v>
       </c>
       <c r="N4" t="n">
-        <v>80.48</v>
+        <v>80.5</v>
       </c>
       <c r="O4" t="n">
-        <v>85.68000000000001</v>
+        <v>85.76000000000001</v>
       </c>
       <c r="P4" t="n">
-        <v>86.40000000000001</v>
+        <v>86.48</v>
       </c>
       <c r="Q4" t="n">
-        <v>92.73999999999999</v>
+        <v>92.81</v>
       </c>
       <c r="R4" t="n">
-        <v>73.52</v>
+        <v>73.65000000000001</v>
       </c>
       <c r="S4" t="n">
-        <v>81.31</v>
+        <v>81.27</v>
       </c>
       <c r="T4" t="n">
         <v>1.311</v>
@@ -798,22 +798,22 @@
         <v>85.23</v>
       </c>
       <c r="N5" t="n">
-        <v>86.95</v>
+        <v>87</v>
       </c>
       <c r="O5" t="n">
-        <v>90.64</v>
+        <v>90.75</v>
       </c>
       <c r="P5" t="n">
-        <v>90.54000000000001</v>
+        <v>90.5</v>
       </c>
       <c r="Q5" t="n">
-        <v>95.11</v>
+        <v>95.14</v>
       </c>
       <c r="R5" t="n">
-        <v>82.29000000000001</v>
+        <v>82.28</v>
       </c>
       <c r="S5" t="n">
-        <v>87.86</v>
+        <v>87.95999999999999</v>
       </c>
       <c r="T5" t="n">
         <v>1.335</v>
@@ -866,22 +866,22 @@
         <v>96.56</v>
       </c>
       <c r="N6" t="n">
-        <v>91.95999999999999</v>
+        <v>92</v>
       </c>
       <c r="O6" t="n">
-        <v>94.7</v>
+        <v>94.73</v>
       </c>
       <c r="P6" t="n">
-        <v>88</v>
+        <v>88.03</v>
       </c>
       <c r="Q6" t="n">
-        <v>92.69</v>
+        <v>92.70999999999999</v>
       </c>
       <c r="R6" t="n">
-        <v>95.13</v>
+        <v>95.20999999999999</v>
       </c>
       <c r="S6" t="n">
-        <v>97.66</v>
+        <v>97.73999999999999</v>
       </c>
       <c r="T6" t="n">
         <v>1.198</v>
@@ -934,22 +934,22 @@
         <v>97.06999999999999</v>
       </c>
       <c r="N7" t="n">
-        <v>92.42</v>
+        <v>92.48</v>
       </c>
       <c r="O7" t="n">
-        <v>94.97</v>
+        <v>95.05</v>
       </c>
       <c r="P7" t="n">
-        <v>88.45</v>
+        <v>88.42</v>
       </c>
       <c r="Q7" t="n">
-        <v>92.84999999999999</v>
+        <v>92.94</v>
       </c>
       <c r="R7" t="n">
-        <v>95.95999999999999</v>
+        <v>95.97</v>
       </c>
       <c r="S7" t="n">
-        <v>98.02</v>
+        <v>98.01000000000001</v>
       </c>
       <c r="T7" t="n">
         <v>1.22</v>
@@ -1002,22 +1002,22 @@
         <v>97.66</v>
       </c>
       <c r="N8" t="n">
-        <v>92.8</v>
+        <v>92.69</v>
       </c>
       <c r="O8" t="n">
-        <v>95.47</v>
+        <v>95.37</v>
       </c>
       <c r="P8" t="n">
         <v>88.41</v>
       </c>
       <c r="Q8" t="n">
-        <v>93.18000000000001</v>
+        <v>93.05</v>
       </c>
       <c r="R8" t="n">
-        <v>96.69</v>
+        <v>96.66</v>
       </c>
       <c r="S8" t="n">
-        <v>98.51000000000001</v>
+        <v>98.48999999999999</v>
       </c>
       <c r="T8" t="n">
         <v>1.233</v>
@@ -1070,22 +1070,22 @@
         <v>96.31999999999999</v>
       </c>
       <c r="N9" t="n">
-        <v>92.01000000000001</v>
+        <v>92.03</v>
       </c>
       <c r="O9" t="n">
-        <v>94.65000000000001</v>
+        <v>94.56</v>
       </c>
       <c r="P9" t="n">
-        <v>88.36</v>
+        <v>88.25</v>
       </c>
       <c r="Q9" t="n">
-        <v>92.77</v>
+        <v>92.67</v>
       </c>
       <c r="R9" t="n">
-        <v>95.04000000000001</v>
+        <v>95.06</v>
       </c>
       <c r="S9" t="n">
-        <v>97.42</v>
+        <v>97.34999999999999</v>
       </c>
       <c r="T9" t="n">
         <v>1.268</v>
@@ -1123,43 +1123,43 @@
         <v>0.25</v>
       </c>
       <c r="I10" t="n">
-        <v>2.202</v>
+        <v>1.752</v>
       </c>
       <c r="J10" t="n">
         <v>1.546</v>
       </c>
       <c r="K10" t="n">
-        <v>65.92</v>
+        <v>73.87</v>
       </c>
       <c r="L10" t="n">
-        <v>59.68</v>
+        <v>74.14</v>
       </c>
       <c r="M10" t="n">
         <v>73.59999999999999</v>
       </c>
       <c r="N10" t="n">
-        <v>63.43</v>
+        <v>71.59</v>
       </c>
       <c r="O10" t="n">
-        <v>68.45999999999999</v>
+        <v>76.03</v>
       </c>
       <c r="P10" t="n">
-        <v>56.26</v>
+        <v>71.18000000000001</v>
       </c>
       <c r="Q10" t="n">
-        <v>63.18</v>
+        <v>76.95999999999999</v>
       </c>
       <c r="R10" t="n">
-        <v>70.11</v>
+        <v>70.18000000000001</v>
       </c>
       <c r="S10" t="n">
-        <v>76.90000000000001</v>
+        <v>76.81</v>
       </c>
       <c r="T10" t="n">
         <v>1.631</v>
       </c>
       <c r="U10" t="n">
-        <v>11971</v>
+        <v>14583</v>
       </c>
     </row>
     <row r="11">
@@ -1191,43 +1191,43 @@
         <v>0.5</v>
       </c>
       <c r="I11" t="n">
-        <v>1.726</v>
+        <v>1.454</v>
       </c>
       <c r="J11" t="n">
         <v>0.751</v>
       </c>
       <c r="K11" t="n">
-        <v>77.42</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="L11" t="n">
-        <v>67.73999999999999</v>
+        <v>80.08</v>
       </c>
       <c r="M11" t="n">
         <v>90.33</v>
       </c>
       <c r="N11" t="n">
-        <v>75.5</v>
+        <v>83.3</v>
       </c>
       <c r="O11" t="n">
-        <v>79.47</v>
+        <v>86.45999999999999</v>
       </c>
       <c r="P11" t="n">
-        <v>64.95</v>
+        <v>77.86</v>
       </c>
       <c r="Q11" t="n">
-        <v>70.56</v>
+        <v>82.05</v>
       </c>
       <c r="R11" t="n">
-        <v>88.03</v>
+        <v>88.17</v>
       </c>
       <c r="S11" t="n">
-        <v>92.48999999999999</v>
+        <v>92.54000000000001</v>
       </c>
       <c r="T11" t="n">
         <v>1.5</v>
       </c>
       <c r="U11" t="n">
-        <v>14404</v>
+        <v>17799</v>
       </c>
     </row>
     <row r="12">
@@ -1259,43 +1259,43 @@
         <v>0.75</v>
       </c>
       <c r="I12" t="n">
-        <v>1.644</v>
+        <v>1.378</v>
       </c>
       <c r="J12" t="n">
         <v>0.577</v>
       </c>
       <c r="K12" t="n">
-        <v>77.65000000000001</v>
+        <v>85.28</v>
       </c>
       <c r="L12" t="n">
-        <v>68.62</v>
+        <v>81.51000000000001</v>
       </c>
       <c r="M12" t="n">
         <v>89.42</v>
       </c>
       <c r="N12" t="n">
-        <v>75.59</v>
+        <v>83.66</v>
       </c>
       <c r="O12" t="n">
-        <v>79.72</v>
+        <v>86.81</v>
       </c>
       <c r="P12" t="n">
-        <v>65.77</v>
+        <v>79.38</v>
       </c>
       <c r="Q12" t="n">
-        <v>71.45999999999999</v>
+        <v>83.51000000000001</v>
       </c>
       <c r="R12" t="n">
-        <v>87.05</v>
+        <v>86.93000000000001</v>
       </c>
       <c r="S12" t="n">
-        <v>91.70999999999999</v>
+        <v>91.73999999999999</v>
       </c>
       <c r="T12" t="n">
         <v>1.482</v>
       </c>
       <c r="U12" t="n">
-        <v>15053</v>
+        <v>18482</v>
       </c>
     </row>
     <row r="13">
@@ -1327,43 +1327,43 @@
         <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>1.673</v>
+        <v>1.4</v>
       </c>
       <c r="J13" t="n">
         <v>0.755</v>
       </c>
       <c r="K13" t="n">
-        <v>77.26000000000001</v>
+        <v>85.95999999999999</v>
       </c>
       <c r="L13" t="n">
-        <v>67.86</v>
+        <v>82.53</v>
       </c>
       <c r="M13" t="n">
         <v>89.68000000000001</v>
       </c>
       <c r="N13" t="n">
-        <v>75.06</v>
+        <v>84.42</v>
       </c>
       <c r="O13" t="n">
-        <v>79.34</v>
+        <v>87.54000000000001</v>
       </c>
       <c r="P13" t="n">
-        <v>64.84999999999999</v>
+        <v>80.45</v>
       </c>
       <c r="Q13" t="n">
-        <v>70.93000000000001</v>
+        <v>84.58</v>
       </c>
       <c r="R13" t="n">
-        <v>87.22</v>
+        <v>87.34</v>
       </c>
       <c r="S13" t="n">
-        <v>91.81999999999999</v>
+        <v>92.03</v>
       </c>
       <c r="T13" t="n">
         <v>1.495</v>
       </c>
       <c r="U13" t="n">
-        <v>15051</v>
+        <v>18934</v>
       </c>
     </row>
     <row r="14">
@@ -1395,43 +1395,43 @@
         <v>0.25</v>
       </c>
       <c r="I14" t="n">
-        <v>2.404</v>
+        <v>2.165</v>
       </c>
       <c r="J14" t="n">
         <v>0.9360000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>76.18000000000001</v>
+        <v>83.45</v>
       </c>
       <c r="L14" t="n">
-        <v>63.57</v>
+        <v>74.37</v>
       </c>
       <c r="M14" t="n">
         <v>95.06</v>
       </c>
       <c r="N14" t="n">
-        <v>74.34</v>
+        <v>82.08</v>
       </c>
       <c r="O14" t="n">
-        <v>78</v>
+        <v>84.77</v>
       </c>
       <c r="P14" t="n">
-        <v>61.12</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="Q14" t="n">
-        <v>65.98999999999999</v>
+        <v>76.31</v>
       </c>
       <c r="R14" t="n">
-        <v>93.56999999999999</v>
+        <v>93.55</v>
       </c>
       <c r="S14" t="n">
-        <v>96.45999999999999</v>
+        <v>96.43000000000001</v>
       </c>
       <c r="T14" t="n">
         <v>1.914</v>
       </c>
       <c r="U14" t="n">
-        <v>35569</v>
+        <v>40947</v>
       </c>
     </row>
     <row r="15">
@@ -1463,34 +1463,34 @@
         <v>0.5</v>
       </c>
       <c r="I15" t="n">
-        <v>2.298</v>
+        <v>1.896</v>
       </c>
       <c r="J15" t="n">
         <v>0.825</v>
       </c>
       <c r="K15" t="n">
-        <v>75.23</v>
+        <v>84.23</v>
       </c>
       <c r="L15" t="n">
-        <v>60.45</v>
+        <v>72.98</v>
       </c>
       <c r="M15" t="n">
         <v>99.56999999999999</v>
       </c>
       <c r="N15" t="n">
-        <v>73.18000000000001</v>
+        <v>82.76000000000001</v>
       </c>
       <c r="O15" t="n">
-        <v>77.14</v>
+        <v>85.64</v>
       </c>
       <c r="P15" t="n">
-        <v>57.83</v>
+        <v>70.78</v>
       </c>
       <c r="Q15" t="n">
-        <v>62.99</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="R15" t="n">
-        <v>99.26000000000001</v>
+        <v>99.23999999999999</v>
       </c>
       <c r="S15" t="n">
         <v>99.83</v>
@@ -1499,7 +1499,7 @@
         <v>1.726</v>
       </c>
       <c r="U15" t="n">
-        <v>28422</v>
+        <v>34804</v>
       </c>
     </row>
     <row r="16">
@@ -1531,34 +1531,34 @@
         <v>0.75</v>
       </c>
       <c r="I16" t="n">
-        <v>2.412</v>
+        <v>1.879</v>
       </c>
       <c r="J16" t="n">
         <v>0.792</v>
       </c>
       <c r="K16" t="n">
-        <v>73.15000000000001</v>
+        <v>85.92</v>
       </c>
       <c r="L16" t="n">
-        <v>57.8</v>
+        <v>75.54000000000001</v>
       </c>
       <c r="M16" t="n">
         <v>99.61</v>
       </c>
       <c r="N16" t="n">
-        <v>71.14</v>
+        <v>84.62</v>
       </c>
       <c r="O16" t="n">
-        <v>75.08</v>
+        <v>87.20999999999999</v>
       </c>
       <c r="P16" t="n">
-        <v>55.34</v>
+        <v>73.56</v>
       </c>
       <c r="Q16" t="n">
-        <v>60.24</v>
+        <v>77.53</v>
       </c>
       <c r="R16" t="n">
-        <v>99.34999999999999</v>
+        <v>99.33</v>
       </c>
       <c r="S16" t="n">
         <v>99.83</v>
@@ -1567,7 +1567,7 @@
         <v>1.748</v>
       </c>
       <c r="U16" t="n">
-        <v>30871</v>
+        <v>41704</v>
       </c>
     </row>
     <row r="17">
@@ -1599,43 +1599,43 @@
         <v>1</v>
       </c>
       <c r="I17" t="n">
-        <v>2.536</v>
+        <v>1.976</v>
       </c>
       <c r="J17" t="n">
         <v>0.661</v>
       </c>
       <c r="K17" t="n">
-        <v>71.81</v>
+        <v>84.03</v>
       </c>
       <c r="L17" t="n">
-        <v>56.11</v>
+        <v>72.62</v>
       </c>
       <c r="M17" t="n">
         <v>99.7</v>
       </c>
       <c r="N17" t="n">
-        <v>69.81999999999999</v>
+        <v>82.79000000000001</v>
       </c>
       <c r="O17" t="n">
-        <v>73.59</v>
+        <v>85.3</v>
       </c>
       <c r="P17" t="n">
-        <v>53.72</v>
+        <v>70.79000000000001</v>
       </c>
       <c r="Q17" t="n">
-        <v>58.35</v>
+        <v>74.54000000000001</v>
       </c>
       <c r="R17" t="n">
-        <v>99.39</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="S17" t="n">
-        <v>99.92</v>
+        <v>99.95999999999999</v>
       </c>
       <c r="T17" t="n">
         <v>1.769</v>
       </c>
       <c r="U17" t="n">
-        <v>39644</v>
+        <v>51047</v>
       </c>
     </row>
     <row r="18">
@@ -1667,34 +1667,34 @@
         <v>0.25</v>
       </c>
       <c r="I18" t="n">
-        <v>2.155</v>
+        <v>1.871</v>
       </c>
       <c r="J18" t="n">
         <v>0.718</v>
       </c>
       <c r="K18" t="n">
-        <v>76.13</v>
+        <v>83.19</v>
       </c>
       <c r="L18" t="n">
-        <v>64.43000000000001</v>
+        <v>75.23999999999999</v>
       </c>
       <c r="M18" t="n">
         <v>93.04000000000001</v>
       </c>
       <c r="N18" t="n">
-        <v>74.2</v>
+        <v>81.69</v>
       </c>
       <c r="O18" t="n">
-        <v>78.04000000000001</v>
+        <v>84.47</v>
       </c>
       <c r="P18" t="n">
-        <v>61.76</v>
+        <v>72.97</v>
       </c>
       <c r="Q18" t="n">
-        <v>67.09999999999999</v>
+        <v>77.17</v>
       </c>
       <c r="R18" t="n">
-        <v>91.40000000000001</v>
+        <v>91.2</v>
       </c>
       <c r="S18" t="n">
         <v>94.66</v>
@@ -1703,7 +1703,7 @@
         <v>1.728</v>
       </c>
       <c r="U18" t="n">
-        <v>42993</v>
+        <v>48544</v>
       </c>
     </row>
     <row r="19">
@@ -1735,43 +1735,43 @@
         <v>0.5</v>
       </c>
       <c r="I19" t="n">
-        <v>2.506</v>
+        <v>2.216</v>
       </c>
       <c r="J19" t="n">
         <v>0.716</v>
       </c>
       <c r="K19" t="n">
-        <v>75.81999999999999</v>
+        <v>84.01000000000001</v>
       </c>
       <c r="L19" t="n">
-        <v>61.71</v>
+        <v>73.36</v>
       </c>
       <c r="M19" t="n">
         <v>98.28</v>
       </c>
       <c r="N19" t="n">
-        <v>74.15000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="O19" t="n">
-        <v>77.42</v>
+        <v>85.12</v>
       </c>
       <c r="P19" t="n">
-        <v>59.56</v>
+        <v>71.7</v>
       </c>
       <c r="Q19" t="n">
-        <v>63.82</v>
+        <v>75.06999999999999</v>
       </c>
       <c r="R19" t="n">
-        <v>97.48</v>
+        <v>97.44</v>
       </c>
       <c r="S19" t="n">
-        <v>98.98999999999999</v>
+        <v>98.95999999999999</v>
       </c>
       <c r="T19" t="n">
         <v>1.929</v>
       </c>
       <c r="U19" t="n">
-        <v>49893</v>
+        <v>57586</v>
       </c>
     </row>
     <row r="20">
@@ -1803,34 +1803,34 @@
         <v>0.75</v>
       </c>
       <c r="I20" t="n">
-        <v>1.878</v>
+        <v>1.61</v>
       </c>
       <c r="J20" t="n">
         <v>0.642</v>
       </c>
       <c r="K20" t="n">
-        <v>80.06999999999999</v>
+        <v>88.48</v>
       </c>
       <c r="L20" t="n">
-        <v>67.17</v>
+        <v>79.92</v>
       </c>
       <c r="M20" t="n">
         <v>99.09999999999999</v>
       </c>
       <c r="N20" t="n">
-        <v>78.25</v>
+        <v>87.27</v>
       </c>
       <c r="O20" t="n">
-        <v>81.75</v>
+        <v>89.62</v>
       </c>
       <c r="P20" t="n">
-        <v>64.63</v>
+        <v>78.01000000000001</v>
       </c>
       <c r="Q20" t="n">
-        <v>69.58</v>
+        <v>81.77</v>
       </c>
       <c r="R20" t="n">
-        <v>98.58</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="S20" t="n">
         <v>99.53</v>
@@ -1839,7 +1839,7 @@
         <v>1.609</v>
       </c>
       <c r="U20" t="n">
-        <v>25986</v>
+        <v>33033</v>
       </c>
     </row>
     <row r="21">
@@ -1871,43 +1871,43 @@
         <v>1</v>
       </c>
       <c r="I21" t="n">
-        <v>2.187</v>
+        <v>1.706</v>
       </c>
       <c r="J21" t="n">
         <v>0.577</v>
       </c>
       <c r="K21" t="n">
-        <v>75.69</v>
+        <v>85.73999999999999</v>
       </c>
       <c r="L21" t="n">
-        <v>61.46</v>
+        <v>75.92</v>
       </c>
       <c r="M21" t="n">
         <v>98.5</v>
       </c>
       <c r="N21" t="n">
-        <v>73.73</v>
+        <v>84.41</v>
       </c>
       <c r="O21" t="n">
-        <v>77.59999999999999</v>
+        <v>87.04000000000001</v>
       </c>
       <c r="P21" t="n">
-        <v>58.91</v>
+        <v>73.87</v>
       </c>
       <c r="Q21" t="n">
-        <v>64.03</v>
+        <v>77.95</v>
       </c>
       <c r="R21" t="n">
         <v>97.83</v>
       </c>
       <c r="S21" t="n">
-        <v>99.11</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="T21" t="n">
         <v>1.644</v>
       </c>
       <c r="U21" t="n">
-        <v>24678</v>
+        <v>32773</v>
       </c>
     </row>
   </sheetData>

</xml_diff>